<commit_message>
update data for peru wtatage and offshore cpue
</commit_message>
<xml_diff>
--- a/assessment/data/SC12_2024assessmentInputData.xlsx
+++ b/assessment/data/SC12_2024assessmentInputData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://southpacificrfmo.sharepoint.com/sites/SPRFMOSCJackMackerelWorkingGroup/Shared Documents/Data repository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="111" documentId="8_{13840C3C-8786-40F8-81E6-DB9B74E4FE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D676794-0F14-4F71-9ED0-1D51DAC96ED9}"/>
+  <xr:revisionPtr revIDLastSave="129" documentId="8_{13840C3C-8786-40F8-81E6-DB9B74E4FE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12D36556-3302-4DC2-BC84-BAAF68D81EAA}"/>
   <bookViews>
-    <workbookView xWindow="1275" yWindow="-120" windowWidth="37245" windowHeight="21840" activeTab="4" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
+    <workbookView xWindow="1275" yWindow="-120" windowWidth="37245" windowHeight="21840" activeTab="3" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
   </bookViews>
   <sheets>
     <sheet name="ageComps" sheetId="1" r:id="rId1"/>
@@ -139,7 +139,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -148,8 +148,6 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -737,7 +735,9 @@
         <v>0</v>
       </c>
       <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
+      <c r="F15" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="1">
@@ -753,7 +753,9 @@
         <v>0</v>
       </c>
       <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
+      <c r="F16" s="1">
+        <v>1396.724070482247</v>
+      </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="1">
@@ -769,7 +771,9 @@
         <v>9194.6801630769223</v>
       </c>
       <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
+      <c r="F17" s="1">
+        <v>2136.4285825586126</v>
+      </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="1">
@@ -785,7 +789,9 @@
         <v>71723.673709753697</v>
       </c>
       <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
+      <c r="F18" s="1">
+        <v>11297.20860288684</v>
+      </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="1">
@@ -801,7 +807,9 @@
         <v>135640.36084989388</v>
       </c>
       <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
+      <c r="F19" s="1">
+        <v>7650.2520916132835</v>
+      </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="1">
@@ -817,7 +825,9 @@
         <v>207312.44981006414</v>
       </c>
       <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
+      <c r="F20" s="1">
+        <v>1916.4894674464028</v>
+      </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="1">
@@ -833,7 +843,9 @@
         <v>161401.39128679619</v>
       </c>
       <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
+      <c r="F21" s="1">
+        <v>526.29527066926426</v>
+      </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="1">
@@ -849,7 +861,9 @@
         <v>87567.333773518636</v>
       </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
+      <c r="F22" s="1">
+        <v>38.636179698004483</v>
+      </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="1">
@@ -865,7 +879,9 @@
         <v>20173.302371896549</v>
       </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
+      <c r="F23" s="1">
+        <v>0.58784683101104662</v>
+      </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="1">
@@ -881,7 +897,9 @@
         <v>4034.6562199999998</v>
       </c>
       <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
+      <c r="F24" s="1">
+        <v>0.58784683101104662</v>
+      </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="1">
@@ -897,7 +915,9 @@
         <v>2376.7831549999996</v>
       </c>
       <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
+      <c r="F25" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="1">
@@ -913,7 +933,9 @@
         <v>45.077870000000004</v>
       </c>
       <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
+      <c r="F26" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="1">
@@ -929,7 +951,9 @@
         <v>0</v>
       </c>
       <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
+      <c r="F27" s="1">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1223,7 +1247,9 @@
         <v>6</v>
       </c>
       <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
+      <c r="F16" s="1">
+        <v>0.19600000000000001</v>
+      </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="1">
@@ -1239,7 +1265,9 @@
         <v>0.29511845898236805</v>
       </c>
       <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
+      <c r="F17" s="1">
+        <v>0.21904316852119662</v>
+      </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="1">
@@ -1255,7 +1283,9 @@
         <v>0.33148786376068634</v>
       </c>
       <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
+      <c r="F18" s="1">
+        <v>0.26719583313830431</v>
+      </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="1">
@@ -1271,7 +1301,9 @@
         <v>0.40214749235203873</v>
       </c>
       <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
+      <c r="F19" s="1">
+        <v>0.46928196931190791</v>
+      </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="1">
@@ -1287,7 +1319,9 @@
         <v>0.49317934331459107</v>
       </c>
       <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
+      <c r="F20" s="1">
+        <v>0.7120412794771328</v>
+      </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="1">
@@ -1303,7 +1337,9 @@
         <v>0.55151009124426742</v>
       </c>
       <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
+      <c r="F21" s="1">
+        <v>0.82109450406118456</v>
+      </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="1">
@@ -1319,7 +1355,9 @@
         <v>0.70050815348785733</v>
       </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
+      <c r="F22" s="1">
+        <v>1.0968487752928646</v>
+      </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="1">
@@ -1335,7 +1373,9 @@
         <v>0.70094952887407047</v>
       </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
+      <c r="F23" s="1">
+        <v>1.131</v>
+      </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="1">
@@ -1351,7 +1391,9 @@
         <v>1.0513357352644144</v>
       </c>
       <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
+      <c r="F24" s="1">
+        <v>1.367</v>
+      </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="1">
@@ -3985,8 +4027,8 @@
       <c r="D40" s="1">
         <v>3.7641645458594568</v>
       </c>
-      <c r="E40">
-        <v>1680</v>
+      <c r="E40" s="1">
+        <v>1653.6802818962401</v>
       </c>
       <c r="H40" s="2"/>
       <c r="J40" s="3"/>
@@ -4001,8 +4043,8 @@
       <c r="D41" s="1">
         <v>1.3242687219012454</v>
       </c>
-      <c r="E41">
-        <v>1185</v>
+      <c r="E41" s="1">
+        <v>1161.92943516948</v>
       </c>
       <c r="H41" s="2"/>
       <c r="J41" s="3"/>
@@ -4017,8 +4059,8 @@
       <c r="D42" s="1">
         <v>2.4500983901372111</v>
       </c>
-      <c r="E42">
-        <v>824</v>
+      <c r="E42" s="1">
+        <v>805.19388247437303</v>
       </c>
       <c r="H42" s="2"/>
       <c r="J42" s="3"/>
@@ -4033,8 +4075,8 @@
       <c r="D43" s="1">
         <v>6.2947270184837389</v>
       </c>
-      <c r="E43">
-        <v>732</v>
+      <c r="E43" s="1">
+        <v>700.19373093011302</v>
       </c>
       <c r="H43" s="2"/>
       <c r="J43" s="3"/>
@@ -4049,8 +4091,8 @@
       <c r="D44" s="1">
         <v>5.4945947291144535</v>
       </c>
-      <c r="E44">
-        <v>618</v>
+      <c r="E44" s="1">
+        <v>596.189979324609</v>
       </c>
       <c r="H44" s="2"/>
       <c r="J44" s="3"/>
@@ -4065,8 +4107,8 @@
       <c r="D45" s="1">
         <v>2.4188396888209356</v>
       </c>
-      <c r="E45">
-        <v>719</v>
+      <c r="E45" s="1">
+        <v>688.01336448665495</v>
       </c>
       <c r="H45" s="2"/>
       <c r="J45" s="3"/>
@@ -4081,8 +4123,8 @@
       <c r="D46" s="1">
         <v>3.2410191810481033</v>
       </c>
-      <c r="E46">
-        <v>760</v>
+      <c r="E46" s="1">
+        <v>725.43112304592296</v>
       </c>
       <c r="H46" s="2"/>
       <c r="J46" s="3"/>
@@ -4097,8 +4139,8 @@
       <c r="D47" s="1">
         <v>2.6219436958550761</v>
       </c>
-      <c r="E47">
-        <v>1035</v>
+      <c r="E47" s="1">
+        <v>967.45742832171095</v>
       </c>
       <c r="H47" s="2"/>
       <c r="J47" s="3"/>
@@ -4113,8 +4155,8 @@
       <c r="D48" s="1">
         <v>2.2360294354738719</v>
       </c>
-      <c r="E48">
-        <v>743</v>
+      <c r="E48" s="1">
+        <v>719.96030790439102</v>
       </c>
       <c r="H48" s="2"/>
       <c r="J48" s="3"/>
@@ -4129,8 +4171,8 @@
       <c r="D49" s="1">
         <v>2.8330904604436409</v>
       </c>
-      <c r="E49">
-        <v>916</v>
+      <c r="E49" s="1">
+        <v>888.37716526156998</v>
       </c>
       <c r="H49" s="2"/>
       <c r="J49" s="3"/>
@@ -4145,8 +4187,8 @@
       <c r="D50" s="1">
         <v>8.119408912961692</v>
       </c>
-      <c r="E50">
-        <v>807</v>
+      <c r="E50" s="1">
+        <v>778.19536234381599</v>
       </c>
       <c r="H50" s="2"/>
       <c r="J50" s="3"/>
@@ -4161,8 +4203,8 @@
       <c r="D51" s="1">
         <v>13.579688603082644</v>
       </c>
-      <c r="E51">
-        <v>975</v>
+      <c r="E51" s="1">
+        <v>923.54846143458894</v>
       </c>
       <c r="H51" s="2"/>
       <c r="J51" s="3"/>
@@ -4177,8 +4219,8 @@
       <c r="D52" s="1">
         <v>14.637762844103841</v>
       </c>
-      <c r="E52">
-        <v>1373</v>
+      <c r="E52" s="1">
+        <v>1242.038753065</v>
       </c>
       <c r="H52" s="2"/>
       <c r="J52" s="3"/>
@@ -4193,8 +4235,8 @@
       <c r="D53" s="1">
         <v>17.77777385219078</v>
       </c>
-      <c r="E53">
-        <v>1714</v>
+      <c r="E53" s="1">
+        <v>1612.9337805719799</v>
       </c>
       <c r="H53" s="2"/>
       <c r="J53" s="3"/>
@@ -4209,8 +4251,8 @@
       <c r="D54" s="1">
         <v>22.304145885248207</v>
       </c>
-      <c r="E54">
-        <v>3032</v>
+      <c r="E54" s="1">
+        <v>2969.7577090576101</v>
       </c>
       <c r="H54" s="2"/>
       <c r="J54" s="3"/>
@@ -4224,6 +4266,9 @@
       </c>
       <c r="D55" s="1">
         <v>22.519976768731979</v>
+      </c>
+      <c r="E55" s="1">
+        <v>1991.15881203303</v>
       </c>
       <c r="H55" s="2"/>
       <c r="J55" s="3"/>
@@ -4272,16 +4317,16 @@
       <c r="A2">
         <v>2023</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="4">
         <v>80466</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="4">
         <v>736292</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="4">
         <v>212119</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="4">
         <v>95334</v>
       </c>
     </row>
@@ -4290,17 +4335,17 @@
         <v>2024</v>
       </c>
       <c r="B3" s="4">
-        <v>67474</v>
+        <v>105727</v>
       </c>
       <c r="C3" s="4">
-        <v>617411</v>
-      </c>
-      <c r="D3" s="5">
-        <v>52324</v>
-      </c>
-      <c r="E3">
-        <f>38400+24000+14805</f>
-        <v>77205</v>
+        <v>855424</v>
+      </c>
+      <c r="D3" s="4">
+        <f>210000+456+25337</f>
+        <v>235793</v>
+      </c>
+      <c r="E3" s="1">
+        <v>68231</v>
       </c>
     </row>
   </sheetData>
@@ -4724,21 +4769,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100812D0B056278C642B7C89719D0EEC9C4" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="53e5abc0267b36fb4b4009f6291778a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f419981a-ca0a-4e56-9512-575f16b7ea2d" xmlns:ns3="5ce05999-5605-4258-98fc-62ff4522b5fb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d299d2548571e9774994fb9c4dbbeb8" ns2:_="" ns3:_="">
     <xsd:import namespace="f419981a-ca0a-4e56-9512-575f16b7ea2d"/>
@@ -4953,24 +4983,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFE542F3-5C46-43FB-860A-90AC96253C26}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4987,4 +5015,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update Chile Acoustic N
</commit_message>
<xml_diff>
--- a/assessment/data/SC12_2024assessmentInputData.xlsx
+++ b/assessment/data/SC12_2024assessmentInputData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://southpacificrfmo.sharepoint.com/sites/SPRFMOSCJackMackerelWorkingGroup/Shared Documents/Data repository/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leeqi/Library/CloudStorage/GoogleDrive-leeqi@uw.edu/My Drive/SPRFMO/jjm/assessment/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="129" documentId="8_{13840C3C-8786-40F8-81E6-DB9B74E4FE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12D36556-3302-4DC2-BC84-BAAF68D81EAA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7D99708-507E-1A40-8BBF-0424009EA296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1275" yWindow="-120" windowWidth="37245" windowHeight="21840" activeTab="3" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
+    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="18880" activeTab="5" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
   </bookViews>
   <sheets>
     <sheet name="ageComps" sheetId="1" r:id="rId1"/>
@@ -83,7 +83,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="##.\ ###"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -465,9 +465,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCC02C38-8F7E-48D4-BE42-B6D35726D79C}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -487,7 +487,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>2023</v>
       </c>
@@ -505,7 +505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2023</v>
       </c>
@@ -523,7 +523,7 @@
         <v>1375.539227616604</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>2023</v>
       </c>
@@ -541,7 +541,7 @@
         <v>51360.56065572107</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>2023</v>
       </c>
@@ -559,7 +559,7 @@
         <v>121217.93615885175</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>2023</v>
       </c>
@@ -577,7 +577,7 @@
         <v>138752.59034703398</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>2023</v>
       </c>
@@ -595,7 +595,7 @@
         <v>27485.728336122211</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>2023</v>
       </c>
@@ -613,7 +613,7 @@
         <v>13618.0873101082</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>2023</v>
       </c>
@@ -631,7 +631,7 @@
         <v>7918.2911239405621</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>2023</v>
       </c>
@@ -649,7 +649,7 @@
         <v>6459.1949629382088</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>2023</v>
       </c>
@@ -667,7 +667,7 @@
         <v>3672.1961122737821</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>2023</v>
       </c>
@@ -685,7 +685,7 @@
         <v>1706.4982771578743</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>2023</v>
       </c>
@@ -703,7 +703,7 @@
         <v>450.76707002476144</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>2023</v>
       </c>
@@ -721,7 +721,7 @@
         <v>353.33421841218382</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>2024</v>
       </c>
@@ -739,7 +739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>2024</v>
       </c>
@@ -757,7 +757,7 @@
         <v>1396.724070482247</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>2024</v>
       </c>
@@ -775,7 +775,7 @@
         <v>2136.4285825586126</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>2024</v>
       </c>
@@ -793,7 +793,7 @@
         <v>11297.20860288684</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>2024</v>
       </c>
@@ -811,7 +811,7 @@
         <v>7650.2520916132835</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>2024</v>
       </c>
@@ -829,7 +829,7 @@
         <v>1916.4894674464028</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>2024</v>
       </c>
@@ -847,7 +847,7 @@
         <v>526.29527066926426</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>2024</v>
       </c>
@@ -865,7 +865,7 @@
         <v>38.636179698004483</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>2024</v>
       </c>
@@ -883,7 +883,7 @@
         <v>0.58784683101104662</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>2024</v>
       </c>
@@ -901,7 +901,7 @@
         <v>0.58784683101104662</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>2024</v>
       </c>
@@ -919,7 +919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>2024</v>
       </c>
@@ -937,7 +937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>2024</v>
       </c>
@@ -963,9 +963,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{209B4BF9-A1A2-42A3-B429-B839E2C11906}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -985,7 +985,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>2023</v>
       </c>
@@ -1001,7 +1001,7 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2023</v>
       </c>
@@ -1019,7 +1019,7 @@
         <v>0.15124242936497981</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>2023</v>
       </c>
@@ -1037,7 +1037,7 @@
         <v>0.18729137695638509</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>2023</v>
       </c>
@@ -1055,7 +1055,7 @@
         <v>0.21142353434513636</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>2023</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>0.22416845405163063</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>2023</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>0.31017208002160995</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>2023</v>
       </c>
@@ -1109,7 +1109,7 @@
         <v>0.39696918996865904</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>2023</v>
       </c>
@@ -1127,7 +1127,7 @@
         <v>0.5125629261211152</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>2023</v>
       </c>
@@ -1145,7 +1145,7 @@
         <v>0.65310069505813761</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>2023</v>
       </c>
@@ -1163,7 +1163,7 @@
         <v>0.75761147312795585</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>2023</v>
       </c>
@@ -1181,7 +1181,7 @@
         <v>0.82092283619174389</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>2023</v>
       </c>
@@ -1199,7 +1199,7 @@
         <v>0.91153912833619943</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>2023</v>
       </c>
@@ -1217,7 +1217,7 @@
         <v>1.1627153380505686</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>2024</v>
       </c>
@@ -1233,7 +1233,7 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>2024</v>
       </c>
@@ -1251,7 +1251,7 @@
         <v>0.19600000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>2024</v>
       </c>
@@ -1269,7 +1269,7 @@
         <v>0.21904316852119662</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>2024</v>
       </c>
@@ -1287,7 +1287,7 @@
         <v>0.26719583313830431</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>2024</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>0.46928196931190791</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>2024</v>
       </c>
@@ -1323,7 +1323,7 @@
         <v>0.7120412794771328</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>2024</v>
       </c>
@@ -1341,7 +1341,7 @@
         <v>0.82109450406118456</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>2024</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>1.0968487752928646</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>2024</v>
       </c>
@@ -1377,7 +1377,7 @@
         <v>1.131</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>2024</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>1.367</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>2024</v>
       </c>
@@ -1411,7 +1411,7 @@
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>2024</v>
       </c>
@@ -1427,7 +1427,7 @@
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>2024</v>
       </c>
@@ -1451,9 +1451,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{045D14A7-CC75-44C0-8FF4-8DE7C82A1AA5}">
   <dimension ref="A1:F201"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1473,7 +1473,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2023</v>
       </c>
@@ -1484,7 +1484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2023</v>
       </c>
@@ -1495,7 +1495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2023</v>
       </c>
@@ -1506,7 +1506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2023</v>
       </c>
@@ -1517,7 +1517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2023</v>
       </c>
@@ -1528,7 +1528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -1539,7 +1539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2023</v>
       </c>
@@ -1550,7 +1550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2023</v>
       </c>
@@ -1561,7 +1561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2023</v>
       </c>
@@ -1572,7 +1572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2023</v>
       </c>
@@ -1583,7 +1583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2023</v>
       </c>
@@ -1594,7 +1594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2023</v>
       </c>
@@ -1605,7 +1605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2023</v>
       </c>
@@ -1616,7 +1616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2023</v>
       </c>
@@ -1627,7 +1627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2023</v>
       </c>
@@ -1638,7 +1638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2023</v>
       </c>
@@ -1649,7 +1649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2023</v>
       </c>
@@ -1660,7 +1660,7 @@
         <v>0.38473646621254598</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2023</v>
       </c>
@@ -1671,7 +1671,7 @@
         <v>3.65589956626388</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>2023</v>
       </c>
@@ -1682,7 +1682,7 @@
         <v>3.210582548075199</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>2023</v>
       </c>
@@ -1693,7 +1693,7 @@
         <v>5.9211604949286949</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>2023</v>
       </c>
@@ -1704,7 +1704,7 @@
         <v>7.5804027299167274</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>2023</v>
       </c>
@@ -1715,7 +1715,7 @@
         <v>24.870441489738365</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>2023</v>
       </c>
@@ -1726,7 +1726,7 @@
         <v>72.532832675437987</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>2023</v>
       </c>
@@ -1737,7 +1737,7 @@
         <v>130.08688029879829</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>2023</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>191.3683053327789</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>2023</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>429.42431713973281</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>2023</v>
       </c>
@@ -1770,7 +1770,7 @@
         <v>790.11558140447164</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>2023</v>
       </c>
@@ -1781,7 +1781,7 @@
         <v>1719.5309159465169</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>2023</v>
       </c>
@@ -1792,7 +1792,7 @@
         <v>3691.0067655112744</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>2023</v>
       </c>
@@ -1803,7 +1803,7 @@
         <v>7223.6098682297661</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>2023</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>12112.870280035952</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>2023</v>
       </c>
@@ -1825,7 +1825,7 @@
         <v>16351.518115564566</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>2023</v>
       </c>
@@ -1836,7 +1836,7 @@
         <v>16273.151532401334</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>2023</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>12946.565903564844</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>2023</v>
       </c>
@@ -1858,7 +1858,7 @@
         <v>10745.534849670372</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>2023</v>
       </c>
@@ -1869,7 +1869,7 @@
         <v>8934.6452316001159</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>2023</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>9443.6721998810644</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>2023</v>
       </c>
@@ -1891,7 +1891,7 @@
         <v>11007.919859757312</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>2023</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>12507.956389445219</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>2023</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>14165.905542779077</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>2023</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>14440.04075624128</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>2023</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>14222.468948530113</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>2023</v>
       </c>
@@ -1946,7 +1946,7 @@
         <v>14098.686846556493</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>2023</v>
       </c>
@@ -1957,7 +1957,7 @@
         <v>13387.579615031149</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>2023</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>13019.475891083417</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>2023</v>
       </c>
@@ -1979,7 +1979,7 @@
         <v>12758.464833698978</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>2023</v>
       </c>
@@ -1990,7 +1990,7 @@
         <v>10907.203998975807</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>2023</v>
       </c>
@@ -2001,7 +2001,7 @@
         <v>9252.2119762584316</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>2023</v>
       </c>
@@ -2012,7 +2012,7 @@
         <v>7321.0266421403549</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>2023</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>5565.8171735107726</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>2023</v>
       </c>
@@ -2034,7 +2034,7 @@
         <v>3797.5084394440269</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>2023</v>
       </c>
@@ -2045,7 +2045,7 @@
         <v>2451.1760363763628</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>2023</v>
       </c>
@@ -2056,7 +2056,7 @@
         <v>1361.8285752782676</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>2023</v>
       </c>
@@ -2067,7 +2067,7 @@
         <v>755.03061172598291</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>2023</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>312.33344587880936</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>2023</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>100.76769342579439</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>2023</v>
       </c>
@@ -2100,7 +2100,7 @@
         <v>52.710601360164318</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>2023</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>17.416527760051839</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>2023</v>
       </c>
@@ -2122,7 +2122,7 @@
         <v>3.338892011033054</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>2023</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>0.1436319092577493</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>2023</v>
       </c>
@@ -2144,7 +2144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>2023</v>
       </c>
@@ -2155,7 +2155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>2023</v>
       </c>
@@ -2166,7 +2166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>2023</v>
       </c>
@@ -2177,7 +2177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>2023</v>
       </c>
@@ -2188,7 +2188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>2023</v>
       </c>
@@ -2199,7 +2199,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>2023</v>
       </c>
@@ -2210,7 +2210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>2023</v>
       </c>
@@ -2221,7 +2221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>2023</v>
       </c>
@@ -2232,7 +2232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:5">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>2023</v>
       </c>
@@ -2243,7 +2243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:5">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>2023</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>2023</v>
       </c>
@@ -2265,7 +2265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:5">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>2023</v>
       </c>
@@ -2276,7 +2276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>2023</v>
       </c>
@@ -2287,7 +2287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>2023</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>2023</v>
       </c>
@@ -2309,7 +2309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>2023</v>
       </c>
@@ -2320,7 +2320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>2023</v>
       </c>
@@ -2331,7 +2331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>2023</v>
       </c>
@@ -2342,7 +2342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>2023</v>
       </c>
@@ -2353,7 +2353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>2023</v>
       </c>
@@ -2364,7 +2364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>2023</v>
       </c>
@@ -2375,7 +2375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>2023</v>
       </c>
@@ -2386,7 +2386,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>2023</v>
       </c>
@@ -2397,7 +2397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:5">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>2023</v>
       </c>
@@ -2408,7 +2408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:5">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>2023</v>
       </c>
@@ -2419,7 +2419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>2023</v>
       </c>
@@ -2430,7 +2430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:5">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>2023</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:5">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>2023</v>
       </c>
@@ -2452,7 +2452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:5">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>2023</v>
       </c>
@@ -2463,7 +2463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:5">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>2023</v>
       </c>
@@ -2474,7 +2474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:5">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>2023</v>
       </c>
@@ -2485,7 +2485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:5">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>2023</v>
       </c>
@@ -2496,7 +2496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:5">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>2023</v>
       </c>
@@ -2507,7 +2507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:5">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>2023</v>
       </c>
@@ -2518,7 +2518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:5">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>2023</v>
       </c>
@@ -2529,7 +2529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:5">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>2023</v>
       </c>
@@ -2540,7 +2540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:5">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>2023</v>
       </c>
@@ -2551,7 +2551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:5">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>2023</v>
       </c>
@@ -2562,7 +2562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:5">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>2023</v>
       </c>
@@ -2573,7 +2573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:5">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>2024</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:5">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>2024</v>
       </c>
@@ -2595,7 +2595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:5">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>2024</v>
       </c>
@@ -2606,7 +2606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:5">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>2024</v>
       </c>
@@ -2617,7 +2617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:5">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>2024</v>
       </c>
@@ -2628,7 +2628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:5">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>2024</v>
       </c>
@@ -2639,7 +2639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:5">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>2024</v>
       </c>
@@ -2650,7 +2650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:5">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>2024</v>
       </c>
@@ -2661,7 +2661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:5">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>2024</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:5">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>2024</v>
       </c>
@@ -2683,7 +2683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:5">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>2024</v>
       </c>
@@ -2694,7 +2694,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:5">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>2024</v>
       </c>
@@ -2705,7 +2705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:5">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>2024</v>
       </c>
@@ -2716,7 +2716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:5">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>2024</v>
       </c>
@@ -2727,7 +2727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:5">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>2024</v>
       </c>
@@ -2738,7 +2738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:5">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>2024</v>
       </c>
@@ -2749,7 +2749,7 @@
         <v>0.83067180597275203</v>
       </c>
     </row>
-    <row r="118" spans="1:5">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>2024</v>
       </c>
@@ -2760,7 +2760,7 @@
         <v>3.16351423658835</v>
       </c>
     </row>
-    <row r="119" spans="1:5">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>2024</v>
       </c>
@@ -2771,7 +2771,7 @@
         <v>1.58891462833298</v>
       </c>
     </row>
-    <row r="120" spans="1:5">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>2024</v>
       </c>
@@ -2782,7 +2782,7 @@
         <v>9.9244160394069905</v>
       </c>
     </row>
-    <row r="121" spans="1:5">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>2024</v>
       </c>
@@ -2793,7 +2793,7 @@
         <v>51.272024610172252</v>
       </c>
     </row>
-    <row r="122" spans="1:5">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>2024</v>
       </c>
@@ -2804,7 +2804,7 @@
         <v>155.6681721266369</v>
       </c>
     </row>
-    <row r="123" spans="1:5">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>2024</v>
       </c>
@@ -2815,7 +2815,7 @@
         <v>207.0955545945817</v>
       </c>
     </row>
-    <row r="124" spans="1:5">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>2024</v>
       </c>
@@ -2826,7 +2826,7 @@
         <v>226.13931360263098</v>
       </c>
     </row>
-    <row r="125" spans="1:5">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>2024</v>
       </c>
@@ -2837,7 +2837,7 @@
         <v>394.03455688927801</v>
       </c>
     </row>
-    <row r="126" spans="1:5">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>2024</v>
       </c>
@@ -2848,7 +2848,7 @@
         <v>626.75134092936003</v>
       </c>
     </row>
-    <row r="127" spans="1:5">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>2024</v>
       </c>
@@ -2859,7 +2859,7 @@
         <v>763.02512816327908</v>
       </c>
     </row>
-    <row r="128" spans="1:5">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>2024</v>
       </c>
@@ -2870,7 +2870,7 @@
         <v>859.40456750131898</v>
       </c>
     </row>
-    <row r="129" spans="1:5">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>2024</v>
       </c>
@@ -2881,7 +2881,7 @@
         <v>724.08464036613702</v>
       </c>
     </row>
-    <row r="130" spans="1:5">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>2024</v>
       </c>
@@ -2892,7 +2892,7 @@
         <v>548.86183415784501</v>
       </c>
     </row>
-    <row r="131" spans="1:5">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>2024</v>
       </c>
@@ -2903,7 +2903,7 @@
         <v>578.95504376725398</v>
       </c>
     </row>
-    <row r="132" spans="1:5">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>2024</v>
       </c>
@@ -2914,7 +2914,7 @@
         <v>592.4877036495725</v>
       </c>
     </row>
-    <row r="133" spans="1:5">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>2024</v>
       </c>
@@ -2925,7 +2925,7 @@
         <v>639.22974953777498</v>
       </c>
     </row>
-    <row r="134" spans="1:5">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>2024</v>
       </c>
@@ -2936,7 +2936,7 @@
         <v>645.88828174250455</v>
       </c>
     </row>
-    <row r="135" spans="1:5">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>2024</v>
       </c>
@@ -2947,7 +2947,7 @@
         <v>633.82032416056893</v>
       </c>
     </row>
-    <row r="136" spans="1:5">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>2024</v>
       </c>
@@ -2958,7 +2958,7 @@
         <v>817.99973166582788</v>
       </c>
     </row>
-    <row r="137" spans="1:5">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>2024</v>
       </c>
@@ -2969,7 +2969,7 @@
         <v>1277.2116540880561</v>
       </c>
     </row>
-    <row r="138" spans="1:5">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>2024</v>
       </c>
@@ -2980,7 +2980,7 @@
         <v>1187.2086678553301</v>
       </c>
     </row>
-    <row r="139" spans="1:5">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>2024</v>
       </c>
@@ -2991,7 +2991,7 @@
         <v>1385.662576527749</v>
       </c>
     </row>
-    <row r="140" spans="1:5">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>2024</v>
       </c>
@@ -3002,7 +3002,7 @@
         <v>1912.756112194523</v>
       </c>
     </row>
-    <row r="141" spans="1:5">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>2024</v>
       </c>
@@ -3013,7 +3013,7 @@
         <v>2237.3885388970548</v>
       </c>
     </row>
-    <row r="142" spans="1:5">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>2024</v>
       </c>
@@ -3024,7 +3024,7 @@
         <v>3037.9025357081582</v>
       </c>
     </row>
-    <row r="143" spans="1:5">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>2024</v>
       </c>
@@ -3035,7 +3035,7 @@
         <v>3955.7731962990706</v>
       </c>
     </row>
-    <row r="144" spans="1:5">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>2024</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>4935.0839096029677</v>
       </c>
     </row>
-    <row r="145" spans="1:5">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>2024</v>
       </c>
@@ -3057,7 +3057,7 @@
         <v>5262.8451463160491</v>
       </c>
     </row>
-    <row r="146" spans="1:5">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>2024</v>
       </c>
@@ -3068,7 +3068,7 @@
         <v>4871.2768547862997</v>
       </c>
     </row>
-    <row r="147" spans="1:5">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>2024</v>
       </c>
@@ -3079,7 +3079,7 @@
         <v>4320.847496610184</v>
       </c>
     </row>
-    <row r="148" spans="1:5">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>2024</v>
       </c>
@@ -3090,7 +3090,7 @@
         <v>3969.415784765692</v>
       </c>
     </row>
-    <row r="149" spans="1:5">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>2024</v>
       </c>
@@ -3101,7 +3101,7 @@
         <v>3844.7901134115282</v>
       </c>
     </row>
-    <row r="150" spans="1:5">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>2024</v>
       </c>
@@ -3112,7 +3112,7 @@
         <v>3630.0971454767823</v>
       </c>
     </row>
-    <row r="151" spans="1:5">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>2024</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>3011.5452672747092</v>
       </c>
     </row>
-    <row r="152" spans="1:5">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152">
         <v>2024</v>
       </c>
@@ -3134,7 +3134,7 @@
         <v>2558.081026167074</v>
       </c>
     </row>
-    <row r="153" spans="1:5">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153">
         <v>2024</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>1773.9519943722557</v>
       </c>
     </row>
-    <row r="154" spans="1:5">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154">
         <v>2024</v>
       </c>
@@ -3156,7 +3156,7 @@
         <v>1179.2282995733694</v>
       </c>
     </row>
-    <row r="155" spans="1:5">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155">
         <v>2024</v>
       </c>
@@ -3167,7 +3167,7 @@
         <v>717.63223684264244</v>
       </c>
     </row>
-    <row r="156" spans="1:5">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A156">
         <v>2024</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>325.46077964969209</v>
       </c>
     </row>
-    <row r="157" spans="1:5">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A157">
         <v>2024</v>
       </c>
@@ -3189,7 +3189,7 @@
         <v>167.53714256785821</v>
       </c>
     </row>
-    <row r="158" spans="1:5">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A158">
         <v>2024</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>52.959066838238201</v>
       </c>
     </row>
-    <row r="159" spans="1:5">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A159">
         <v>2024</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>4.6508754190266801</v>
       </c>
     </row>
-    <row r="160" spans="1:5">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A160">
         <v>2024</v>
       </c>
@@ -3222,7 +3222,7 @@
         <v>0.63547056525420598</v>
       </c>
     </row>
-    <row r="161" spans="1:5">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A161">
         <v>2024</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:5">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A162">
         <v>2024</v>
       </c>
@@ -3244,7 +3244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:5">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A163">
         <v>2024</v>
       </c>
@@ -3255,7 +3255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:5">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A164">
         <v>2024</v>
       </c>
@@ -3266,7 +3266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:5">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A165">
         <v>2024</v>
       </c>
@@ -3277,7 +3277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:5">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>2024</v>
       </c>
@@ -3288,7 +3288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:5">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A167">
         <v>2024</v>
       </c>
@@ -3299,7 +3299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:5">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A168">
         <v>2024</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:5">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A169">
         <v>2024</v>
       </c>
@@ -3321,7 +3321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:5">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A170">
         <v>2024</v>
       </c>
@@ -3332,7 +3332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:5">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A171">
         <v>2024</v>
       </c>
@@ -3343,7 +3343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:5">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A172">
         <v>2024</v>
       </c>
@@ -3354,7 +3354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:5">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A173">
         <v>2024</v>
       </c>
@@ -3365,7 +3365,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:5">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A174">
         <v>2024</v>
       </c>
@@ -3376,7 +3376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:5">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A175">
         <v>2024</v>
       </c>
@@ -3387,7 +3387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:5">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A176">
         <v>2024</v>
       </c>
@@ -3398,7 +3398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:5">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A177">
         <v>2024</v>
       </c>
@@ -3409,7 +3409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:5">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A178">
         <v>2024</v>
       </c>
@@ -3420,7 +3420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:5">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A179">
         <v>2024</v>
       </c>
@@ -3431,7 +3431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:5">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A180">
         <v>2024</v>
       </c>
@@ -3442,7 +3442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:5">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A181">
         <v>2024</v>
       </c>
@@ -3453,7 +3453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:5">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A182">
         <v>2024</v>
       </c>
@@ -3464,7 +3464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:5">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A183">
         <v>2024</v>
       </c>
@@ -3475,7 +3475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:5">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A184">
         <v>2024</v>
       </c>
@@ -3486,7 +3486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:5">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A185">
         <v>2024</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:5">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A186">
         <v>2024</v>
       </c>
@@ -3508,7 +3508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:5">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A187">
         <v>2024</v>
       </c>
@@ -3519,7 +3519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:5">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A188">
         <v>2024</v>
       </c>
@@ -3530,7 +3530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:5">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A189">
         <v>2024</v>
       </c>
@@ -3541,7 +3541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:5">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A190">
         <v>2024</v>
       </c>
@@ -3552,7 +3552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:5">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A191">
         <v>2024</v>
       </c>
@@ -3563,7 +3563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:5">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A192">
         <v>2024</v>
       </c>
@@ -3574,7 +3574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:5">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A193">
         <v>2024</v>
       </c>
@@ -3585,7 +3585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:5">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A194">
         <v>2024</v>
       </c>
@@ -3596,7 +3596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:5">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A195">
         <v>2024</v>
       </c>
@@ -3607,7 +3607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:5">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A196">
         <v>2024</v>
       </c>
@@ -3618,7 +3618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:5">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A197">
         <v>2024</v>
       </c>
@@ -3629,7 +3629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:5">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A198">
         <v>2024</v>
       </c>
@@ -3640,7 +3640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:5">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A199">
         <v>2024</v>
       </c>
@@ -3651,7 +3651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:5">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A200">
         <v>2024</v>
       </c>
@@ -3662,7 +3662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:5">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A201">
         <v>2024</v>
       </c>
@@ -3681,9 +3681,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7886E624-8038-4FB5-9240-586936FC87C7}">
   <dimension ref="A1:J56"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3700,73 +3700,73 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1970</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1971</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1972</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1973</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1974</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1975</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1976</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1977</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>1978</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>1979</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>1980</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>1981</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>1982</v>
       </c>
       <c r="C14" s="1"/>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>1983</v>
       </c>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>1984</v>
       </c>
@@ -3784,7 +3784,7 @@
       </c>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>1985</v>
       </c>
@@ -3793,7 +3793,7 @@
       </c>
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>1986</v>
       </c>
@@ -3802,7 +3802,7 @@
       </c>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>1987</v>
       </c>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>1988</v>
       </c>
@@ -3820,7 +3820,7 @@
       </c>
       <c r="H20" s="2"/>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>1989</v>
       </c>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="H21" s="2"/>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>1990</v>
       </c>
@@ -3838,7 +3838,7 @@
       </c>
       <c r="H22" s="2"/>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>1991</v>
       </c>
@@ -3847,7 +3847,7 @@
       </c>
       <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>1992</v>
       </c>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>1993</v>
       </c>
@@ -3865,7 +3865,7 @@
       </c>
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>1994</v>
       </c>
@@ -3874,7 +3874,7 @@
       </c>
       <c r="H26" s="2"/>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>1995</v>
       </c>
@@ -3883,7 +3883,7 @@
       </c>
       <c r="H27" s="2"/>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>1996</v>
       </c>
@@ -3892,7 +3892,7 @@
       </c>
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>1997</v>
       </c>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>1998</v>
       </c>
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H30" s="2"/>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>1999</v>
       </c>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>2000</v>
       </c>
@@ -3929,7 +3929,7 @@
       <c r="D32" s="1"/>
       <c r="H32" s="2"/>
     </row>
-    <row r="33" spans="1:10">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>2001</v>
       </c>
@@ -3939,7 +3939,7 @@
       <c r="D33" s="1"/>
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="1:10">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>2002</v>
       </c>
@@ -3952,7 +3952,7 @@
       <c r="H34" s="2"/>
       <c r="J34" s="3"/>
     </row>
-    <row r="35" spans="1:10">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>2003</v>
       </c>
@@ -3965,7 +3965,7 @@
       <c r="H35" s="2"/>
       <c r="J35" s="3"/>
     </row>
-    <row r="36" spans="1:10">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>2004</v>
       </c>
@@ -3978,7 +3978,7 @@
       <c r="H36" s="2"/>
       <c r="J36" s="3"/>
     </row>
-    <row r="37" spans="1:10">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>2005</v>
       </c>
@@ -3991,7 +3991,7 @@
       <c r="H37" s="2"/>
       <c r="J37" s="3"/>
     </row>
-    <row r="38" spans="1:10">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>2006</v>
       </c>
@@ -4004,7 +4004,7 @@
       <c r="H38" s="2"/>
       <c r="J38" s="3"/>
     </row>
-    <row r="39" spans="1:10">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>2007</v>
       </c>
@@ -4017,7 +4017,7 @@
       <c r="H39" s="2"/>
       <c r="J39" s="3"/>
     </row>
-    <row r="40" spans="1:10">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>2008</v>
       </c>
@@ -4033,7 +4033,7 @@
       <c r="H40" s="2"/>
       <c r="J40" s="3"/>
     </row>
-    <row r="41" spans="1:10">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>2009</v>
       </c>
@@ -4049,7 +4049,7 @@
       <c r="H41" s="2"/>
       <c r="J41" s="3"/>
     </row>
-    <row r="42" spans="1:10">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>2010</v>
       </c>
@@ -4065,7 +4065,7 @@
       <c r="H42" s="2"/>
       <c r="J42" s="3"/>
     </row>
-    <row r="43" spans="1:10">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>2011</v>
       </c>
@@ -4081,7 +4081,7 @@
       <c r="H43" s="2"/>
       <c r="J43" s="3"/>
     </row>
-    <row r="44" spans="1:10">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>2012</v>
       </c>
@@ -4097,7 +4097,7 @@
       <c r="H44" s="2"/>
       <c r="J44" s="3"/>
     </row>
-    <row r="45" spans="1:10">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>2013</v>
       </c>
@@ -4113,7 +4113,7 @@
       <c r="H45" s="2"/>
       <c r="J45" s="3"/>
     </row>
-    <row r="46" spans="1:10">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>2014</v>
       </c>
@@ -4129,7 +4129,7 @@
       <c r="H46" s="2"/>
       <c r="J46" s="3"/>
     </row>
-    <row r="47" spans="1:10">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>2015</v>
       </c>
@@ -4145,7 +4145,7 @@
       <c r="H47" s="2"/>
       <c r="J47" s="3"/>
     </row>
-    <row r="48" spans="1:10">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>2016</v>
       </c>
@@ -4161,7 +4161,7 @@
       <c r="H48" s="2"/>
       <c r="J48" s="3"/>
     </row>
-    <row r="49" spans="1:10">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>2017</v>
       </c>
@@ -4177,7 +4177,7 @@
       <c r="H49" s="2"/>
       <c r="J49" s="3"/>
     </row>
-    <row r="50" spans="1:10">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>2018</v>
       </c>
@@ -4193,7 +4193,7 @@
       <c r="H50" s="2"/>
       <c r="J50" s="3"/>
     </row>
-    <row r="51" spans="1:10">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>2019</v>
       </c>
@@ -4209,7 +4209,7 @@
       <c r="H51" s="2"/>
       <c r="J51" s="3"/>
     </row>
-    <row r="52" spans="1:10">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>2020</v>
       </c>
@@ -4225,7 +4225,7 @@
       <c r="H52" s="2"/>
       <c r="J52" s="3"/>
     </row>
-    <row r="53" spans="1:10">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>2021</v>
       </c>
@@ -4241,7 +4241,7 @@
       <c r="H53" s="2"/>
       <c r="J53" s="3"/>
     </row>
-    <row r="54" spans="1:10">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>2022</v>
       </c>
@@ -4257,7 +4257,7 @@
       <c r="H54" s="2"/>
       <c r="J54" s="3"/>
     </row>
-    <row r="55" spans="1:10">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>2023</v>
       </c>
@@ -4273,7 +4273,7 @@
       <c r="H55" s="2"/>
       <c r="J55" s="3"/>
     </row>
-    <row r="56" spans="1:10">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>2024</v>
       </c>
@@ -4294,9 +4294,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA686FE5-9B92-4435-B67D-4EE55A2A4B01}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4313,7 +4313,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2023</v>
       </c>
@@ -4330,7 +4330,7 @@
         <v>95334</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2024</v>
       </c>
@@ -4356,9 +4356,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E42CCE45-3DDC-4861-A006-F4C4C7145E6D}">
   <dimension ref="A1:G27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4381,7 +4381,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -4391,12 +4391,10 @@
       <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="1">
-        <v>2250643.7089896626</v>
-      </c>
+      <c r="D2" s="1"/>
       <c r="E2" s="1"/>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2024</v>
       </c>
@@ -4407,11 +4405,11 @@
         <v>9</v>
       </c>
       <c r="D3" s="1">
-        <v>6724033.3132093837</v>
+        <v>8974677.0221990459</v>
       </c>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2024</v>
       </c>
@@ -4426,7 +4424,7 @@
       </c>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2024</v>
       </c>
@@ -4441,7 +4439,7 @@
       </c>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2024</v>
       </c>
@@ -4456,7 +4454,7 @@
       </c>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2024</v>
       </c>
@@ -4471,7 +4469,7 @@
       </c>
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -4486,7 +4484,7 @@
       </c>
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2024</v>
       </c>
@@ -4501,7 +4499,7 @@
       </c>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2024</v>
       </c>
@@ -4516,7 +4514,7 @@
       </c>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2024</v>
       </c>
@@ -4531,7 +4529,7 @@
       </c>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2024</v>
       </c>
@@ -4546,7 +4544,7 @@
       </c>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2024</v>
       </c>
@@ -4559,7 +4557,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2024</v>
       </c>
@@ -4572,7 +4570,7 @@
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2024</v>
       </c>
@@ -4582,12 +4580,10 @@
       <c r="C15" t="s">
         <v>10</v>
       </c>
-      <c r="D15" s="1">
-        <v>4.6398307123951668E-2</v>
-      </c>
+      <c r="D15" s="1"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2024</v>
       </c>
@@ -4598,11 +4594,11 @@
         <v>10</v>
       </c>
       <c r="D16" s="1">
-        <v>7.1104990245594274E-2</v>
+        <v>6.5053084042619863E-2</v>
       </c>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2024</v>
       </c>
@@ -4617,7 +4613,7 @@
       </c>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2024</v>
       </c>
@@ -4632,7 +4628,7 @@
       </c>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2024</v>
       </c>
@@ -4647,7 +4643,7 @@
       </c>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>2024</v>
       </c>
@@ -4662,7 +4658,7 @@
       </c>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>2024</v>
       </c>
@@ -4677,7 +4673,7 @@
       </c>
       <c r="E21" s="1"/>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>2024</v>
       </c>
@@ -4692,7 +4688,7 @@
       </c>
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>2024</v>
       </c>
@@ -4707,7 +4703,7 @@
       </c>
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>2024</v>
       </c>
@@ -4722,7 +4718,7 @@
       </c>
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>2024</v>
       </c>
@@ -4737,7 +4733,7 @@
       </c>
       <c r="E25" s="1"/>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>2024</v>
       </c>
@@ -4750,7 +4746,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>2024</v>
       </c>
@@ -4769,6 +4765,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100812D0B056278C642B7C89719D0EEC9C4" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="53e5abc0267b36fb4b4009f6291778a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f419981a-ca0a-4e56-9512-575f16b7ea2d" xmlns:ns3="5ce05999-5605-4258-98fc-62ff4522b5fb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d299d2548571e9774994fb9c4dbbeb8" ns2:_="" ns3:_="">
     <xsd:import namespace="f419981a-ca0a-4e56-9512-575f16b7ea2d"/>
@@ -4983,12 +4985,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -4999,6 +4995,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFE542F3-5C46-43FB-860A-90AC96253C26}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5017,15 +5022,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
update with new data
</commit_message>
<xml_diff>
--- a/assessment/data/SC12_2024assessmentInputData.xlsx
+++ b/assessment/data/SC12_2024assessmentInputData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leeqi/Library/CloudStorage/GoogleDrive-leeqi@uw.edu/My Drive/SPRFMO/jjm/assessment/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7D99708-507E-1A40-8BBF-0424009EA296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51646EE5-69C6-B141-9A30-06C6AB827B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="18880" activeTab="5" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
+    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="18880" activeTab="1" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
   </bookViews>
   <sheets>
     <sheet name="ageComps" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="11">
   <si>
     <t>year</t>
   </si>
@@ -154,7 +154,22 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{AC837FF7-52FA-4EFD-8030-01534540C025}"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="gray0625">
+          <fgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray0625">
+          <fgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -494,9 +509,7 @@
       <c r="B2" s="1">
         <v>0</v>
       </c>
-      <c r="C2" s="1">
-        <v>9248.8443894663706</v>
-      </c>
+      <c r="C2" s="1"/>
       <c r="D2" s="1">
         <v>0</v>
       </c>
@@ -513,7 +526,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="1">
-        <v>0</v>
+        <v>9248.8443894663706</v>
       </c>
       <c r="D3" s="1">
         <v>149.197</v>
@@ -992,9 +1005,7 @@
       <c r="B2" s="1">
         <v>0</v>
       </c>
-      <c r="C2" s="1">
-        <v>1.0179991360722711E-2</v>
-      </c>
+      <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
@@ -1008,8 +1019,8 @@
       <c r="B3" s="1">
         <v>1</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>6</v>
+      <c r="C3" s="1">
+        <v>1.0179991360722711E-2</v>
       </c>
       <c r="D3" s="1">
         <v>0.19600000000000001</v>
@@ -4324,7 +4335,7 @@
         <v>736292</v>
       </c>
       <c r="D2" s="4">
-        <v>212119</v>
+        <v>222287</v>
       </c>
       <c r="E2" s="4">
         <v>95334</v>
@@ -4765,9 +4776,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4986,19 +5000,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5023,9 +5033,10 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update to catch data
</commit_message>
<xml_diff>
--- a/assessment/data/SC12_2024assessmentInputData.xlsx
+++ b/assessment/data/SC12_2024assessmentInputData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leeqi/Library/CloudStorage/GoogleDrive-leeqi@uw.edu/My Drive/SPRFMO/jjm/assessment/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51646EE5-69C6-B141-9A30-06C6AB827B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A772FC7C-06F7-C842-9A75-75F989F5E272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="18880" activeTab="1" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
+    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="18880" activeTab="4" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
   </bookViews>
   <sheets>
     <sheet name="ageComps" sheetId="1" r:id="rId1"/>
@@ -154,22 +154,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{AC837FF7-52FA-4EFD-8030-01534540C025}"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill patternType="gray0625">
-          <fgColor theme="0" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray0625">
-          <fgColor theme="0" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -4329,10 +4314,10 @@
         <v>2023</v>
       </c>
       <c r="B2" s="4">
-        <v>80466</v>
+        <v>68052</v>
       </c>
       <c r="C2" s="4">
-        <v>736292</v>
+        <v>740203</v>
       </c>
       <c r="D2" s="4">
         <v>222287</v>
@@ -4776,6 +4761,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -4784,7 +4775,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100812D0B056278C642B7C89719D0EEC9C4" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="53e5abc0267b36fb4b4009f6291778a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f419981a-ca0a-4e56-9512-575f16b7ea2d" xmlns:ns3="5ce05999-5605-4258-98fc-62ff4522b5fb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d299d2548571e9774994fb9c4dbbeb8" ns2:_="" ns3:_="">
     <xsd:import namespace="f419981a-ca0a-4e56-9512-575f16b7ea2d"/>
@@ -4999,13 +4990,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -5013,7 +5007,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFE542F3-5C46-43FB-860A-90AC96253C26}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5030,13 +5024,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>